<commit_message>
feat: add optional onsite reception codes
</commit_message>
<xml_diff>
--- a/학교 연수 전자서명 시스템 - 배포용 원본.xlsx
+++ b/학교 연수 전자서명 시스템 - 배포용 원본.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📘 사용설명서" sheetId="1" r:id="R22398b158c734fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📘 사용설명서" sheetId="1" r:id="R20213cef86c242cc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1488,7 +1488,7 @@
       </x:c>
       <x:c r="D26" s="32" t="str">
         <x:v>연수에서 날짜·시간·활성 상태와 서명 대상(전체 구성원 또는 부서 선택)을 정합니다.
-참고  선택한 부서에 나중에 추가되는 구성원도 자동으로 대상에 포함됩니다. 지난 연수도 활성화하면 재수합할 수 있습니다.</x:v>
+참고  필요한 연수에만 현장 접수 코드 사용을 켭니다. 기존 연수와 이 항목을 끈 연수는 코드 없이 운영됩니다.</x:v>
       </x:c>
       <x:c r="E26" s="109"/>
       <x:c r="F26" s="3"/>
@@ -1538,11 +1538,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C30" s="66" t="str">
-        <x:v>참여 화면 점검</x:v>
+        <x:v>현장 접수와 참여</x:v>
       </x:c>
       <x:c r="D30" s="32" t="str">
-        <x:v>연수 날짜·시간·활성 상태를 확인하고 공유 링크를 휴대폰에서도 열어 봅니다.
-참고  참여자는 연수 선택 → 본인 선택 → 서명 제출 순서로 진행합니다.</x:v>
+        <x:v>현장 코드 연수는 카드에서 5·10·15분 접수를 열고 화면의 6자리 코드를 현장에서 안내합니다.
+참고  재발급·종료 시 이전 코드는 즉시 무효화되며, 오늘·매일 연수는 등록된 종료 시각에 맞춰 접수도 끝납니다.</x:v>
       </x:c>
       <x:c r="E30" s="109"/>
       <x:c r="F30" s="3"/>

</xml_diff>

<commit_message>
Protect owner email in deployment guide
</commit_message>
<xml_diff>
--- a/학교 연수 전자서명 시스템 - 배포용 원본.xlsx
+++ b/학교 연수 전자서명 시스템 - 배포용 원본.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📘 사용설명서" sheetId="1" r:id="R55ad3386aa4c4ece"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📘 사용설명서" sheetId="1" r:id="R5514eb3040864bbe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -571,11 +571,11 @@
       </x:c>
       <x:c r="D8" s="20" t="str">
         <x:v>새 사본에서 🖊️ 전자서명 관리 → 초기 설정 실행을 누르고, 완료 창의 초기 설정 코드를 보관합니다.
-참고  ‘Google에서 확인하지 않은 앱’이 나오면 개발자 이메일이 본인 계정인지 확인한 뒤 고급 → 학교 연수 전자서명 시스템으로 이동 → 허용을 누릅니다. 모르는 이메일이거나 Google Workspace 정책이 차단하면 중단하고 관리자에게 문의하세요. 소유자만 처음 한 번 승인하며 서명 참여자에게는 이 화면이 나타나지 않습니다.</x:v>
+참고  ‘Google에서 확인하지 않은 앱’이 나오면 이 사본을 만든 본인 Google 계정으로 로그인했는지 확인한 뒤 고급 → 학교 연수 전자서명 시스템으로 이동 → 허용을 누릅니다. 본인이 만들지 않은 사본이거나 Google Workspace 정책이 차단하면 중단하고 관리자에게 문의하세요. 사본 소유자만 처음 한 번 승인하며 서명 참여자에게는 이 화면이 나타나지 않습니다.</x:v>
       </x:c>
       <x:c r="E8" s="20" t="str">
         <x:v>새 사본에서 🖊️ 전자서명 관리 → 초기 설정 실행을 누르고, 완료 창의 초기 설정 코드를 보관합니다.
-참고  ‘Google에서 확인하지 않은 앱’이 나오면 개발자 이메일이 본인 계정인지 확인한 뒤 고급 → 학교 연수 전자서명 시스템으로 이동 → 허용을 누릅니다. 모르는 이메일이거나 Google Workspace 정책이 차단하면 중단하고 관리자에게 문의하세요. 소유자만 처음 한 번 승인하며 서명 참여자에게는 이 화면이 나타나지 않습니다.</x:v>
+참고  ‘Google에서 확인하지 않은 앱’이 나오면 이 사본을 만든 본인 Google 계정으로 로그인했는지 확인한 뒤 고급 → 학교 연수 전자서명 시스템으로 이동 → 허용을 누릅니다. 본인이 만들지 않은 사본이거나 Google Workspace 정책이 차단하면 중단하고 관리자에게 문의하세요. 사본 소유자만 처음 한 번 승인하며 서명 참여자에게는 이 화면이 나타나지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="90" customHeight="1">

</xml_diff>